<commit_message>
#45 Client BOM updated, minor changes in Gerber. Files ready to release.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v2.1/BOM/Client-BOM-IoT-Button-v2.1.xlsx
+++ b/Design Files/IoT-Button-v2.1/BOM/Client-BOM-IoT-Button-v2.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v2.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="128">
   <si>
     <t>#</t>
   </si>
@@ -394,13 +394,22 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>5V - 2A, Barrel Connector, Polarity Center Positive, Size: OD 5.5mm, ID 2.6mm, Insertion depth 8.3mm</t>
+  </si>
+  <si>
+    <t>Please verify barrel plug dimensions at the time of ordering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,6 +464,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -575,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -612,9 +628,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -622,6 +635,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -911,7 +930,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -935,9 +954,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1429,28 +1448,28 @@
       <c r="C17" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="I17" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="J17" s="15">
+      <c r="J17" s="14">
         <v>1</v>
       </c>
-      <c r="K17" s="17" t="s">
+      <c r="K17" s="16" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1677,6 +1696,38 @@
         <v>1</v>
       </c>
       <c r="K24" s="9"/>
+    </row>
+    <row r="25" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="11">
+        <v>23</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>127</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>